<commit_message>
Update normalized KangaLife club bookings file and remove temporary backup
</commit_message>
<xml_diff>
--- a/web-development/sem1-break-homework/normalised_kangalife_club_bookings_august_2026.xlsx
+++ b/web-development/sem1-break-homework/normalised_kangalife_club_bookings_august_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keyme\repos\Diploma-IT-Course-Work\web-development\sem1-break-homework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B2832395-7BD2-4477-B530-D753EA12C255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{009FAAD8-C786-4860-A0EE-EFF00402FBA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{B0753A72-7664-4DBB-BC9C-71B5D6AFD8AB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{B0753A72-7664-4DBB-BC9C-71B5D6AFD8AB}"/>
   </bookViews>
   <sheets>
     <sheet name="bookings" sheetId="1" r:id="rId1"/>
@@ -748,6 +748,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1242,9 +1245,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1292,7 +1295,7 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1301,7 +1304,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="27" formatCode="d/mm/yyyy\ h:mm"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1362,10 +1365,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2FB49D73-889A-4A2D-AC37-F5A2CECABB6E}" name="Table4_1" displayName="Table4_1" ref="A1:D37" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D37" xr:uid="{2FB49D73-889A-4A2D-AC37-F5A2CECABB6E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{491417CF-1526-40F8-A76E-F00515642458}" uniqueName="1" name="member_id" queryTableFieldId="1" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{A5825E30-7210-404B-AB92-0FA60E9846CB}" uniqueName="2" name="name" queryTableFieldId="2" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{F6852AD0-53FC-4BF4-84EF-1547C8327A7E}" uniqueName="3" name="date_of_birth" queryTableFieldId="3" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{C28459F6-29B5-4285-9749-F8FFD9F4B3ED}" uniqueName="4" name="member_level" queryTableFieldId="4" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{491417CF-1526-40F8-A76E-F00515642458}" uniqueName="1" name="member_id" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{A5825E30-7210-404B-AB92-0FA60E9846CB}" uniqueName="2" name="name" queryTableFieldId="2" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{F6852AD0-53FC-4BF4-84EF-1547C8327A7E}" uniqueName="3" name="date_of_birth" queryTableFieldId="3" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{C28459F6-29B5-4285-9749-F8FFD9F4B3ED}" uniqueName="4" name="member_level" queryTableFieldId="4" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1702,7 +1705,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1714,7 +1717,7 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -1723,7 +1726,7 @@
       <c r="G1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="I1" t="s">
@@ -5518,7 +5521,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B1" t="s">
@@ -5756,18 +5759,18 @@
   <cols>
     <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
       <c r="B1" t="s">
         <v>234</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D1" t="s">
@@ -5781,7 +5784,7 @@
       <c r="B2" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="6">
         <v>20293</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -5795,7 +5798,7 @@
       <c r="B3" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="6">
         <v>23816</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -5809,7 +5812,7 @@
       <c r="B4" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <v>38511</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -5823,7 +5826,7 @@
       <c r="B5" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="6">
         <v>32106</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -5837,7 +5840,7 @@
       <c r="B6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="6">
         <v>39713</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -5851,7 +5854,7 @@
       <c r="B7" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="6">
         <v>27966</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -5865,7 +5868,7 @@
       <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="6">
         <v>31527</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -5879,7 +5882,7 @@
       <c r="B9" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="6">
         <v>21879</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -5893,7 +5896,7 @@
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="6">
         <v>38968</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -5907,7 +5910,7 @@
       <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="6">
         <v>24171</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -5921,7 +5924,7 @@
       <c r="B12" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="6">
         <v>37964</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -5935,7 +5938,7 @@
       <c r="B13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="6">
         <v>19852</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -5949,7 +5952,7 @@
       <c r="B14" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="6">
         <v>20775</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -5963,7 +5966,7 @@
       <c r="B15" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="6">
         <v>38223</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -5977,7 +5980,7 @@
       <c r="B16" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="6">
         <v>22860</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -5991,7 +5994,7 @@
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="6">
         <v>19675</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -6005,7 +6008,7 @@
       <c r="B18" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="6">
         <v>34127</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -6019,7 +6022,7 @@
       <c r="B19" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="6">
         <v>36014</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -6033,7 +6036,7 @@
       <c r="B20" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="6">
         <v>24765</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -6047,7 +6050,7 @@
       <c r="B21" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="6">
         <v>37207</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -6061,7 +6064,7 @@
       <c r="B22" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="6">
         <v>36446</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -6075,7 +6078,7 @@
       <c r="B23" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="6">
         <v>25934</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -6089,7 +6092,7 @@
       <c r="B24" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="6">
         <v>19771</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -6103,7 +6106,7 @@
       <c r="B25" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="6">
         <v>37961</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -6117,7 +6120,7 @@
       <c r="B26" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="6">
         <v>39666</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -6131,7 +6134,7 @@
       <c r="B27" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C27" s="4">
+      <c r="C27" s="6">
         <v>36656</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -6145,7 +6148,7 @@
       <c r="B28" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="6">
         <v>39017</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -6159,7 +6162,7 @@
       <c r="B29" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C29" s="4">
+      <c r="C29" s="6">
         <v>21151</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -6173,7 +6176,7 @@
       <c r="B30" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="6">
         <v>21877</v>
       </c>
       <c r="D30" s="3" t="s">
@@ -6187,7 +6190,7 @@
       <c r="B31" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="6">
         <v>26312</v>
       </c>
       <c r="D31" s="3" t="s">
@@ -6201,7 +6204,7 @@
       <c r="B32" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="6">
         <v>31782</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -6215,7 +6218,7 @@
       <c r="B33" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="6">
         <v>29777</v>
       </c>
       <c r="D33" s="3" t="s">
@@ -6229,7 +6232,7 @@
       <c r="B34" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="4">
+      <c r="C34" s="6">
         <v>25356</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -6243,7 +6246,7 @@
       <c r="B35" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C35" s="4">
+      <c r="C35" s="6">
         <v>38639</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -6257,7 +6260,7 @@
       <c r="B36" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="4">
+      <c r="C36" s="6">
         <v>35929</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -6271,7 +6274,7 @@
       <c r="B37" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="4">
+      <c r="C37" s="6">
         <v>34339</v>
       </c>
       <c r="D37" s="3" t="s">

</xml_diff>